<commit_message>
Sustitución de BMP085 por DHT11, adición de zumbador horario y registro de Max/Min
</commit_message>
<xml_diff>
--- a/docs/conexiones.xlsx
+++ b/docs/conexiones.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juan\Desktop\antigravity\uno+tft\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juan\Desktop\antigravity\uno+tft\reloj_sd\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A703D14C-232F-4C5B-9899-1C967F5401BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4CECED3-AACD-484D-B97D-E00D2FCBF6A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="1770" windowWidth="29040" windowHeight="16440" xr2:uid="{60665AAD-2805-435D-A9C9-0BB50882B3ED}"/>
+    <workbookView xWindow="11820" yWindow="2445" windowWidth="21600" windowHeight="11835" xr2:uid="{60665AAD-2805-435D-A9C9-0BB50882B3ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,18 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="75">
   <si>
     <t>Este proyecto usa un reloj externo (DS1307/DS3231) y un sensor BMP085.</t>
   </si>
   <si>
     <t>Función</t>
-  </si>
-  <si>
-    <t>A4</t>
-  </si>
-  <si>
-    <t>A5</t>
   </si>
   <si>
     <t>TIP</t>
@@ -293,6 +287,9 @@
       </rPr>
       <t>)</t>
     </r>
+  </si>
+  <si>
+    <t>Pin en Arduino Mega</t>
   </si>
 </sst>
 </file>
@@ -909,14 +906,14 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A1" s="22" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A2" s="23" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -940,7 +937,7 @@
     </row>
     <row r="6" spans="1:5" ht="21" x14ac:dyDescent="0.25">
       <c r="A6" s="24" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -952,7 +949,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -964,7 +961,7 @@
     </row>
     <row r="10" spans="1:5" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="20" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -976,10 +973,10 @@
     </row>
     <row r="12" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>1</v>
@@ -989,65 +986,65 @@
     </row>
     <row r="13" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="13" t="s">
         <v>17</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>19</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
     <row r="14" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="13" t="s">
         <v>20</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>22</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="13" t="s">
         <v>23</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>25</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>26</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>28</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
     </row>
     <row r="17" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="16" t="s">
         <v>29</v>
-      </c>
-      <c r="B17" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>31</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
@@ -1059,7 +1056,7 @@
     </row>
     <row r="19" spans="1:5" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A19" s="20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
@@ -1071,97 +1068,97 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
     </row>
     <row r="22" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
     </row>
     <row r="23" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
     </row>
     <row r="24" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
     </row>
     <row r="25" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
     </row>
     <row r="26" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
     </row>
     <row r="27" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
     </row>
     <row r="28" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
     </row>
     <row r="29" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
     </row>
     <row r="30" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
@@ -1173,7 +1170,7 @@
     </row>
     <row r="32" spans="1:5" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="20" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
@@ -1185,10 +1182,10 @@
     </row>
     <row r="34" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C34" s="10" t="s">
         <v>1</v>
@@ -1198,52 +1195,52 @@
     </row>
     <row r="35" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C35" s="13" t="s">
         <v>51</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>53</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
     </row>
     <row r="36" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C36" s="13" t="s">
         <v>54</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>56</v>
       </c>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
     </row>
     <row r="37" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C37" s="13" t="s">
         <v>57</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C37" s="13" t="s">
-        <v>59</v>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
     </row>
     <row r="38" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C38" s="16" t="s">
         <v>60</v>
-      </c>
-      <c r="B38" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="C38" s="16" t="s">
-        <v>62</v>
       </c>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
@@ -1255,7 +1252,7 @@
     </row>
     <row r="40" spans="1:5" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A40" s="20" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
@@ -1267,17 +1264,17 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
     </row>
     <row r="43" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>16</v>
+        <v>74</v>
       </c>
       <c r="C43" s="10" t="s">
         <v>1</v>
@@ -1287,58 +1284,58 @@
     </row>
     <row r="44" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="B44" s="12" t="s">
-        <v>2</v>
+        <v>64</v>
+      </c>
+      <c r="B44" s="12">
+        <v>20</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
     </row>
     <row r="45" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="B45" s="12" t="s">
-        <v>3</v>
+        <v>66</v>
+      </c>
+      <c r="B45" s="12">
+        <v>21</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="11" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B46" s="12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="C47" s="16" t="s">
         <v>72</v>
-      </c>
-      <c r="B47" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="C47" s="16" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A48" s="19" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
@@ -1346,7 +1343,7 @@
     </row>
     <row r="51" spans="1:1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A51" s="22" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
@@ -1354,17 +1351,17 @@
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
@@ -1372,7 +1369,7 @@
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>